<commit_message>
Update master ETL data
</commit_message>
<xml_diff>
--- a/master_etl.xlsx
+++ b/master_etl.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V262"/>
+  <dimension ref="A1:V263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25586,6 +25586,102 @@
       <c r="V262" t="inlineStr">
         <is>
           <t>Economics (Business Economics and Business Innovation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>273</v>
+      </c>
+      <c r="B263" t="n">
+        <v>2</v>
+      </c>
+      <c r="C263" t="n">
+        <v>2568</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Ms.</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>mondog</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>joe</t>
+        </is>
+      </c>
+      <c r="G263" s="1" t="n">
+        <v>37120</v>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Student (Currently studying)</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>No. 34, Zhoujiatun, Chaoge Village, Longyan Township, Huanjiang Maonan Autonomous County, Guangxi, China</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>Guangxi Arts University</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>College of Music</t>
+        </is>
+      </c>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>Master of Music (Music) (Revised version 2023) Plan A (A2)</t>
+        </is>
+      </c>
+      <c r="O263" s="1" t="n">
+        <v>45889</v>
+      </c>
+      <c r="P263" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>20-29</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="S263" t="n">
+        <v>2025</v>
+      </c>
+      <c r="T263" t="n">
+        <v>8</v>
+      </c>
+      <c r="U263" t="inlineStr">
+        <is>
+          <t>August</t>
+        </is>
+      </c>
+      <c r="V263" t="inlineStr">
+        <is>
+          <t>Music (Music)</t>
         </is>
       </c>
     </row>
@@ -25916,7 +26012,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>int32</t>
+          <t>int64</t>
         </is>
       </c>
     </row>

</xml_diff>